<commit_message>
Added a logout button to  guest guest_dashboard
</commit_message>
<xml_diff>
--- a/Documentation.xlsx
+++ b/Documentation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Djando Projects\Hotel_management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9745DD9A-7873-4B6F-8155-2EB81882D3EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C15E70-765F-4AF7-AE66-91E9594C4542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{49060195-078E-40AC-8EF3-DC123239AA5D}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="57">
   <si>
     <t>Python</t>
   </si>
@@ -261,6 +261,13 @@
   <si>
     <t>*Create views and databse for it
 *Test if it works</t>
+  </si>
+  <si>
+    <t>*10:30 - Started working on writing this.
+*16:30 - Finished prototype of Login module, Testing is fine.</t>
+  </si>
+  <si>
+    <t>*No logout function in dashboard template so logout wont work even though the backend is there.</t>
   </si>
 </sst>
 </file>
@@ -683,6 +690,12 @@
       <c r="D2" s="2" t="s">
         <v>48</v>
       </c>
+      <c r="E2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">

</xml_diff>